<commit_message>
Clarify MR lessons, Wegovy PDFs, Drive setup and Sheets workflow
</commit_message>
<xml_diff>
--- a/manager/종근당_MR_거래처목록.xlsx
+++ b/manager/종근당_MR_거래처목록.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="거래처목록" sheetId="1" r:id="R9bce4350be474744"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성예시" sheetId="2" r:id="R0cef4a98f7fe4908"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="월별매출" sheetId="3" r:id="Rb331c5e5a5164604"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="매출요약" sheetId="4" r:id="R18553754d61c462d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="거래처목록" sheetId="1" r:id="Rbbf349ce3454443c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성예시" sheetId="2" r:id="Re445f7b8ccf246d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="월별매출" sheetId="3" r:id="R8c3b3ea01c374090"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="매출요약" sheetId="4" r:id="R60b47765df124e31"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -650,7 +650,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>기관명·의료진명이 같은 대상은 한 행. 사용 제품은 확인된 것만 기록. 매출은 월별매출 시트에 입력합니다.</x:v>
+        <x:v>엑셀은 배포 양식입니다. Drive 업로드 후 파일 → Google Sheets로 저장하세요. 실제 기록은 변환된 Google Sheets의 거래처목록 탭에 입력합니다. 작성예시는 참고용입니다.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -1051,7 +1051,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb11154e94b7a467f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a06bd9d19dc4e41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1095,7 +1095,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>기관명·의료진명이 같은 대상은 한 행. 사용 제품은 확인된 것만 기록. 매출은 월별매출 시트에 입력합니다.</x:v>
+        <x:v>엑셀은 배포 양식입니다. Drive 업로드 후 파일 → Google Sheets로 저장하세요. 실제 기록은 변환된 Google Sheets의 거래처목록 탭에 입력합니다. 작성예시는 참고용입니다.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -1171,65 +1171,59 @@
     </x:row>
     <x:row r="5" ht="64" customHeight="1">
       <x:c r="A5" s="12" t="str">
-        <x:v>대한내과</x:v>
+        <x:v>연세원내과</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>김민국</x:v>
+        <x:v>박정환</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
         <x:v>내과</x:v>
       </x:c>
-      <x:c r="D5" s="14"/>
-      <x:c r="E5" s="14" t="n">
-        <x:v>46311</x:v>
+      <x:c r="D5" s="14" t="str"/>
+      <x:c r="E5" s="14" t="d">
+        <x:v>2026-10-16T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
-        <x:v>골다공증·denosumab</x:v>
+        <x:v>비만·위고비</x:v>
       </x:c>
       <x:c r="G5" s="12" t="str">
-        <x:v>마케팅 제공 근거 확인본</x:v>
+        <x:v>위고비 논문</x:v>
       </x:c>
       <x:c r="H5" s="12" t="str">
         <x:v>미전달</x:v>
       </x:c>
       <x:c r="I5" s="12" t="str">
-        <x:v>근거 대상·한계 확인</x:v>
+        <x:v>위고비 논문 자료 미전달</x:v>
       </x:c>
       <x:c r="J5" s="12" t="str">
-        <x:v>논문 확인 후 재방문 준비</x:v>
+        <x:v>마케팅 자료 확인 후 연구 대상·한계 정리</x:v>
       </x:c>
       <x:c r="K5" s="12" t="str">
-        <x:v>2026-10-23 15:00~15:15 Asia/Seoul</x:v>
-      </x:c>
-      <x:c r="L5" s="12"/>
+        <x:v>2026-10-23 15:00~15:15 Asia/Seoul / Calendar 미등록</x:v>
+      </x:c>
+      <x:c r="L5" s="12" t="str"/>
       <x:c r="M5" s="12" t="str">
-        <x:v>대한내과_김민국_기록.txt</x:v>
+        <x:v>연세원내과_박정환_기록.txt</x:v>
       </x:c>
       <x:c r="N5" s="64" t="str">
-        <x:v>대한내과_김민국_20261016_면담.txt</x:v>
+        <x:v>연세원내과_박정환_20261016_면담.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="64" customHeight="1">
-      <x:c r="A6" s="13" t="str">
-        <x:v>무궁정형외과</x:v>
-      </x:c>
-      <x:c r="B6" s="13" t="str">
-        <x:v>정태백</x:v>
-      </x:c>
-      <x:c r="C6" s="13" t="str">
-        <x:v>정형외과</x:v>
-      </x:c>
-      <x:c r="D6" s="15"/>
-      <x:c r="E6" s="15"/>
-      <x:c r="F6" s="13"/>
-      <x:c r="G6" s="13"/>
-      <x:c r="H6" s="13"/>
-      <x:c r="I6" s="13"/>
-      <x:c r="J6" s="13"/>
-      <x:c r="K6" s="13"/>
-      <x:c r="L6" s="13"/>
-      <x:c r="M6" s="13"/>
-      <x:c r="N6" s="64"/>
+      <x:c r="A6" s="13" t="str"/>
+      <x:c r="B6" s="13" t="str"/>
+      <x:c r="C6" s="13" t="str"/>
+      <x:c r="D6" s="15" t="str"/>
+      <x:c r="E6" s="15" t="str"/>
+      <x:c r="F6" s="13" t="str"/>
+      <x:c r="G6" s="13" t="str"/>
+      <x:c r="H6" s="13" t="str"/>
+      <x:c r="I6" s="13" t="str"/>
+      <x:c r="J6" s="13" t="str"/>
+      <x:c r="K6" s="13" t="str"/>
+      <x:c r="L6" s="13" t="str"/>
+      <x:c r="M6" s="13" t="str"/>
+      <x:c r="N6" s="64" t="str"/>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
       <x:c r="A7" s="12"/>
@@ -1526,7 +1520,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68b33237e9794a5a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ed8257d1b024c6f"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>